<commit_message>
Book 2 quick reference, decision tools and templates aligned with Model v0.8
Operational collection rate vs PAYGo PERFORM 2026 KPIs (T05 gains a
PERFORM_2026 sheet with numerator/denominator check); T01 memo shows the
evidence-based readiness decision beside the recommendation, provenance and
the IFRS statement; T02 adds a PERFORM item and a red flag; 'Lender view'
replaces the bankability step; source statuses (ESMAP pending, M-KOPA
conflicting, BBOXX pending); Book 2 branding; version 0.9 (pre-release).
All rebuilt workbooks recalculated in LibreOffice without errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192koLK9F8fRH5Bfqszi1tY
</commit_message>
<xml_diff>
--- a/volumes/02-solar-home-systems/decision-tools/AEF_V2_D1_Price_Plan_and_APR_Calculator.xlsx
+++ b/volumes/02-solar-home-systems/decision-tools/AEF_V2_D1_Price_Plan_and_APR_Calculator.xlsx
@@ -569,7 +569,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AFRICA ENERGY FINANCE  |  VOLUME 2  |  SOLAR HOME SYSTEMS</t>
+          <t>AFRICA ENERGY FINANCE  |  BOOK 2  |  PAYGO SOLAR FINANCE</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -605,7 +605,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Decision tool D1  |  Version 1.0  |  Author &amp; ideation: Emmanuel Boujieka Kamga</t>
+          <t>Decision tool D1  |  Version 0.9 (pre-release)  |  Author &amp; ideation: Emmanuel Boujieka Kamga</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
@@ -738,7 +738,7 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Links to the Volume 2 model and book</t>
+          <t>Links to Book 2 and MODEL 2</t>
         </is>
       </c>
       <c r="B21" s="6" t="n"/>
@@ -809,7 +809,7 @@
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;"Arial"&amp;8 Africa Energy Finance | Volume 2 Decision tool D1&amp;C&amp;"Arial"&amp;8 &amp;A&amp;R&amp;"Arial"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Arial"&amp;8 Africa Energy Finance | Book 2 Decision tool D1 | Version 0.9 (pre-release)&amp;C&amp;"Arial"&amp;8 &amp;A&amp;R&amp;"Arial"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -840,7 +840,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AFRICA ENERGY FINANCE  |  VOLUME 2  |  SOLAR HOME SYSTEMS</t>
+          <t>AFRICA ENERGY FINANCE  |  BOOK 2  |  PAYGO SOLAR FINANCE</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -882,7 +882,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Decision tool D1  |  Version 1.0  |  Author &amp; ideation: Emmanuel Boujieka Kamga</t>
+          <t>Decision tool D1  |  Version 0.9 (pre-release)  |  Author &amp; ideation: Emmanuel Boujieka Kamga</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
@@ -1821,7 +1821,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;"Arial"&amp;8 Africa Energy Finance | Volume 2 Decision tool D1&amp;C&amp;"Arial"&amp;8 &amp;A&amp;R&amp;"Arial"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Arial"&amp;8 Africa Energy Finance | Book 2 Decision tool D1 | Version 0.9 (pre-release)&amp;C&amp;"Arial"&amp;8 &amp;A&amp;R&amp;"Arial"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>